<commit_message>
Upload para o novo repositorio porto
</commit_message>
<xml_diff>
--- a/Arquivos_CTP/dados_acareacoes_CTP.xlsx
+++ b/Arquivos_CTP/dados_acareacoes_CTP.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,12 +466,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3320084479112</t>
+          <t>3320024958404</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Karina Liege Carvalho</t>
+          <t>(CTG LOC)LINCOWN LUIS(NOVO)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -481,44 +481,44 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Maria Cecília Avelar</t>
+          <t>Dauane Marques Marques</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>+5531997651393</t>
+          <t>+5531971905590</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Rua Joana escolástica rosa 73 Esquina do sinal Casa branca, Betim</t>
+          <t>Rua Nova Friburgo 28 casa, Contagem</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Calca Cargo Jeans Feminina Plus size com lycra*1</t>
+          <t>1 PECA Top Faixa Sem Costura – Sutiã Invisível que Não Marca a Roupa*1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>5.78</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-06-09 14:41:10</t>
+          <t>2026-09-11 11:43:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>3320048502658</t>
+          <t>3320006940844</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>(CTG LOC)Junior Gonçalves</t>
+          <t>(LOC CTG) ANDREIA MARQUES BRAGA (NOVO)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -528,44 +528,44 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Gabii Cordeiro375</t>
+          <t>Alma rica</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>+5531975211860</t>
+          <t>+5531991385105</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Avenida Doutor José Mariano 820 Loja 2, Betim</t>
+          <t>Avenida Alvarenga Peixoto 597, Contagem</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CONJUNTO ESPORTIVO FEMININO DE ALCA CINTURA ALTA CANELADA SEM DETALHE DE COSTURA HZ014*1</t>
+          <t>CroquiChic Body Manga Longa com Dedeira e Recorte Frontal Estilo Gringa*1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>5.66</t>
+          <t>8.08</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-06-09 13:28:18</t>
+          <t>2026-09-11 11:42:38</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3320072504124</t>
+          <t>3320032941862</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>(CTG LOC) Wendel Welberth Sousa Aurelino</t>
+          <t>Janaina Santos (SAULO)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -575,44 +575,44 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ana Cristina Quintal</t>
+          <t>Luziane Karine</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+5531985849985</t>
+          <t>+5538998250799</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Rua Dezesseis 597 casa, Contagem</t>
+          <t>Rua Joaquim José 577 apt402 bl 01, Contagem</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Kit Placas Ripados Decorativo Adesiva 45x11 Painel Premium De Alta Qualidade Sala Penteadeira*1</t>
+          <t>Macacão Feminino Pantalona com bojo Cintura Alta Elegante Verão Casual Chic com Bolso*1</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>129.4</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-06-09 13:28:12</t>
+          <t>2026-09-11 11:42:36</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3320027506836</t>
+          <t>3320049948662</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>(CTG LOC) Wendel Welberth Sousa Aurelino</t>
+          <t>(CTG LOC)Lucas Henrique Caetan Silvestre</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -622,44 +622,44 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ray Ray</t>
+          <t>Joyce Peixoto</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>+5531991293568</t>
+          <t>+5531993926073</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Rua Mônaco 35 casa 02, Contagem</t>
+          <t>Rua Dom Geraldo Fernandes Bijos 900, Contagem</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Camiseta 100% Algodão BK Cantor DLRE Abebe Bikila Streetwear Harajuku Aesthetic Camisa Unissex*1</t>
+          <t>Kit Crochê Completo 53 Peças Para Fazer Amigurumi Agulhas Cabo Soft Tesoura Acessórios Lar Das Fitas Marcadores Estojo*1</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>19.99</t>
+          <t>6.34</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-06-09 13:27:33</t>
+          <t>2026-09-11 11:42:21</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3320083494067</t>
+          <t>3320071914388</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>(CTG LOC) Wendel Welberth Sousa Aurelino</t>
+          <t>(CTG LOC) Marya Eduarda de Costro(John)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -669,44 +669,44 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Michele Pereira alves</t>
+          <t>Fernanda</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>+5531986360591</t>
+          <t>+5531987663218</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Rua Sequóia 594, Contagem</t>
+          <t>Rua Wilson Gramiscelli 50 Apto 304 Bloco 3, Contagem</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Atualizado Projetor Smart HY 300 Android Full HD 1920x1080 Bluetooth Wi-fi*1</t>
+          <t>Kit C/3 Sutiã Básico Com Bojo Do P Ao Gg Direto da Fábrica Escolha Cor*1</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>15.85</t>
+          <t>34.99</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-06-09 13:27:31</t>
+          <t>2026-09-11 11:42:12</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3320060498630</t>
+          <t>3320060945363</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>(CTG INT)Daniele Celestino Leal(Joaquim)</t>
+          <t>(CTG LOC) JOHN HELBERT (NOVO)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -716,44 +716,44 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CARLA Andrea Almeida carneiro indio</t>
+          <t>Jonatan Chagas</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>+5531983866133</t>
+          <t>+5521965515488</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Avenida Amor-Perfeito 275, Betim</t>
+          <t>Rua Eucalípto 75 Apto 303, Contagem</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Lip Balm Bálsamo Labial hidratante Proteção dos Lábios À Prova D'água Batom de mudança de cor hidratação duradoura*1</t>
+          <t>Caneta De Reparo De Pintura De Carro À Prova D'água Transparente Removedor De Arranhões Cores Variadas*1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0.93</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-06-09 13:27:23</t>
+          <t>2026-09-11 11:42:04</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3320044500560</t>
+          <t>3320081910083</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>(CTG LOC) Wendel Welberth Sousa Aurelino</t>
+          <t>(LOC CTG) ANDREIA MARQUES BRAGA (NOVO)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -763,44 +763,44 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Aurecy de Jesus Rocha Novaes</t>
+          <t>Reinaldo Martins</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>+5531992694305</t>
+          <t>+5531997242830</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Rua Vinte e Um 120 apartamento 102 bloco 03, Contagem</t>
+          <t>GF peças diesel 763 loja, Contagem</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Varal De Chão Com Abas Slim Em Aço Reforçado*1</t>
+          <t>Luva Escova Tira Pelos True Touch para Cães e Gatos com Pontas de Silicone*1</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>28.99</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-06-09 13:27:11</t>
+          <t>2026-09-11 11:41:58</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3320023507605</t>
+          <t>3320020949393</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>(CTG LOC)ROGERIO RAMOS DOS SANTOS(NOVO)</t>
+          <t>(LOC CTG) VALDINEY DA SILVA (NOVO)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -810,44 +810,44 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Mariana da Cruz</t>
+          <t>Keyssy Lucas</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>+5531998190812</t>
+          <t>+5531975696899</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Rua do Melão 275 bloco 02, apto 302, Contagem</t>
+          <t>Rua Joaquim Ferreira de Barros 49 galpao, Contagem</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Babuche Sandália Infantil Menino Astronauta Foguete Papete Personalizada Confortável Antiderrapante Detalhe Lateral*1</t>
+          <t>Kit 3 Camiseta Feminina Plus Size Instalando Shape Academia Streetwear Camisa Algodão 26.1 Premium*1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>14.85</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-06-09 13:26:36</t>
+          <t>2026-09-11 11:41:56</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3320017506677</t>
+          <t>3320044947610</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>(CTG LOC) Wendel Welberth Sousa Aurelino</t>
+          <t>(CTG LOC) Tulio Henrique Batista Alves</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -857,44 +857,44 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Gabriela de Paula</t>
+          <t>Ana Clara</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>+5531992679704</t>
+          <t>+5531998229283</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Avenida João Gomes Cardoso 2088 Depósito de construção, Contagem</t>
+          <t>Avenida Rio Negro 1222 Bloco 6 apto 201, Contagem</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Calça Legging Flare Flanelada Leg Boca De Sino Bailarina Grossa Zero Transparência Cintura Alta Confortável Fitness Apertado*1</t>
+          <t>Limpador Magnético De Vidros Aquários Janelas Limpeza Vidro*1</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>4.01</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-06-09 13:26:35</t>
+          <t>2026-09-11 11:41:22</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3320080493611</t>
+          <t>3320053937664</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>(CTG LOC) Wendel Welberth Sousa Aurelino</t>
+          <t>(CTG LOC) WENDEL WELBERTH</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -904,44 +904,44 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Michele Pereira alves</t>
+          <t>Janainefonseca</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>+5531986360591</t>
+          <t>+5538997540712</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Rua Sequóia 594, Contagem</t>
+          <t>Rua Macaúbas 855 Casa, Contagem</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>BETTDOW Tela de projeção antirreflexo cinza de 100-120 polegadas 16:9 para home theater interno e externo | Acessório portátil dobrável*1</t>
+          <t>X55 Fone TWS Sem Fio Alta Performance Conexão Rápida Bluetooth Display LED Preciso Som Estéreo HIFI Cristalino Conforto Total Sem Desconforto Auricular Especial Para Dormir*1</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>0.49</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-06-09 13:26:00</t>
+          <t>2026-09-11 11:40:42</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3320085491582</t>
+          <t>3320062945493</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>(CTG LOC)RODOLFO RODRIGUES(NOVO)</t>
+          <t>(LOC CTG) GUILHERME SALA NOBREGA (NOVO)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -951,44 +951,44 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Maria Betania</t>
+          <t>Raffaely Silva</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>+5531984086913</t>
+          <t>+5531989156141</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Rua Inglaterra/ caso esteja fechado deixar no motel. 797, Contagem</t>
+          <t>Avenida Alterosa 1035, Contagem</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Óleo Rosa Mosqueta 100% Puro e Natural | Rosa Rubiginosa | Clareia Manchas e Estrias | Pura Botânica Óleo Firmador Corporal Óleo De Alta Qualidade*1</t>
+          <t>Porta Papel Higiênico Matelado C/ Aplicação e Aviamento Para 3 Rolos*1</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>13.9</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-06-09 13:25:37</t>
+          <t>2026-09-11 11:39:36</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3320081504505</t>
+          <t>3320070941074</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>(CTG LOC)LINCOWN LUIS(NOVO)</t>
+          <t>(LOC CTG) ELOI DOMINGOS BRAGA (NOVO)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -998,44 +998,44 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Jennifer Gonçalves</t>
+          <t>Thais</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>+5531975286638</t>
+          <t>+5531992151707</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Rua São Benedito 123 portao cinza bater forte, Contagem</t>
+          <t>Rua Gerônimo Soares Barbosa 38 Casa, Contagem</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Durag Silky Waves Bandana Hip Hop Preta Branca Azul Vermelha Compressão 360*1</t>
+          <t>1 Amor Coração Luxo Camurça Caso De Couro Para iPhone 17 16 11 12 13 14 15 Pro Max Plus XR X XS Capa Macia*1</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>2.53</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-06-09 10:53:05</t>
+          <t>2026-09-11 09:56:14</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3320041504730</t>
+          <t>3320053835074</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>(CTG LOC) Raphael de Oliveira Soares</t>
+          <t>(LOC CTG) VILSON JUNIO VIANA (NOVO)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1045,44 +1045,44 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>faela12344566</t>
+          <t>Deliana Bueno</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>+5531995831793</t>
+          <t>+5531992455853</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Rua VL - 35 88 perto supercado campo sa, Contagem</t>
+          <t>Rua das Sempre-Vivas 181 Apartamento 404 bloco 7, Contagem</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Cinta Modeladora Feminina Redutora Abdominal/Afina a Cintura/Fitness*1</t>
+          <t>Ventilador de Teto LED 2 em 1 120W Bivolt 52cm com Controle Remoto*1</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-06-09 10:53:00</t>
+          <t>2026-09-10 13:37:27</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3320002514420</t>
+          <t>3320054947826</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>(CTG LOC) Wendel Welberth Sousa Aurelino</t>
+          <t>(LOC CTG) ELOI DOMINGOS BRAGA (NOVO)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1092,44 +1092,44 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Vitória Emanuele</t>
+          <t>Isabella Chagas de Magalhães</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>+5531989131034</t>
+          <t>+5553199122079</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Rua Imbuia 791, Contagem</t>
+          <t>Rua três 297 202, Contagem</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Kit Médica Maleta, Infantil, Educativo, Divertido, Brinquedo Menina, Mini Doutora, Rosa 14 Peças*1</t>
+          <t>9 Em 1 Escova De Limpeza Elétrica Recarregável Sem Fio 25W Potente Para Limpeza Doméstica E Automotiva Com 2000mAh E Rotação 360°*1</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>13.9</t>
+          <t>6.68</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-06-09 10:52:43</t>
+          <t>2026-09-10 13:35:57</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3320072490213</t>
+          <t>3320077917508</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>(CTG LOC) Wendel Welberth Sousa Aurelino</t>
+          <t>(CTG LOC)EDUARDO DE ASSIS(NOVO)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1139,44 +1139,44 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Rosana de Oliveira</t>
+          <t>Tatiana Carla</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>+5531989154866</t>
+          <t>+5531984112476</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Rua Ímola 01, Contagem</t>
+          <t>Rua Santa Terezinha 325 portão verde claro, Contagem</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>KIT COM 10 PEÇAS CABECEIRA + PLACAS MDF PARA CAMAS KING , QUEEN E SOLTEIRO – KIT DECORATIVO*1</t>
+          <t>Pote Hermético Vidro 320/640ml/1520ml Jogo de Mantimentos Para Cozinha Marmitas Com Travas Freezer Microondas Fitness*1</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>3.43</t>
+          <t>15.59</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-06-09 10:52:38</t>
+          <t>2026-09-10 13:33:26</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3320089503202</t>
+          <t>3320083916641</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>(CTG LOC) Ana Cristina Ferreira(Felipe)</t>
+          <t>(LOC CTG) EVERTON MARTINS SOUZA (NOVO)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1186,44 +1186,44 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Taynara Bragança</t>
+          <t>Angelo da Silva</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>+5531975382167</t>
+          <t>+5531998260235</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Rua Professora Dahir Diniz 781, Contagem</t>
+          <t>Rua José Mendes Ferreira 829 A, Contagem</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Espelho De Maquiagem Para Viseira Solar De Carro , Com 3 Modos De Luz LED , Tela Sensível Ao Toque Regulável , Interior*1</t>
+          <t>Meião de Futebol Longo Antiderrapante Jcolour | Par Único com Solado de Borracha e Tecido Respirável (Tam 40-46)*1</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>1.48</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-06-09 09:51:49</t>
+          <t>2026-09-10 12:14:40</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3320080500759</t>
+          <t>3320091933934</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>(CTG LOC) Wendel Welberth Sousa Aurelino</t>
+          <t>(CTG LOC) Willian Cesar Galdino Santos</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1233,44 +1233,44 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Carlos Ercílio</t>
+          <t>Juliana Flávia Silva</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>+5531975638336</t>
+          <t>+5531995646978</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Rua Caviúna 376, Contagem</t>
+          <t>Rua Osvaldo Cruz 242, Contagem</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Perfume Arabe Eau De Perfume Al Wataniah Eternal Zaeem Unissex 100ml*1</t>
+          <t>calça femenina elegante cintura alta en alfaiataria*1</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>4.78</t>
+          <t>38.37</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-06-09 09:26:01</t>
+          <t>2026-09-10 12:14:23</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3320051482070</t>
+          <t>3320027936100</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>(CTG INT) Vitor G N D Carmo(MATHEUS)</t>
+          <t>(CTG LOC)WANDERSON MARTINS(NOVO)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1280,44 +1280,44 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Karine rosely</t>
+          <t>iza</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>+5531995200390</t>
+          <t>+5531971060203</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Avenida Juiz Marco Túlio Isaac 1119 Quiosque new case, Betim</t>
+          <t>Rua Dolomita 112, Contagem</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Um conjunto com 10 pincéis de maquiagem profissionais*1+Bolsa Organizadora De Joias Portátil , Estojo De Armazenamento Para Colares , Brincos , Organizador*1</t>
+          <t>Piercing Argola Compatível Com Umbigo Aço Cirúgico Pvd Clik 1 Fileira Zircônia Piercing de Umbigo Argola*1</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>0.47</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-06-08 14:24:54</t>
+          <t>2026-09-10 12:12:53</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3320019505507</t>
+          <t>3320038941966</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>(CTG LOC)Junior Gonçalves</t>
+          <t>(LOC CTG) ANDREIA MARQUES BRAGA (NOVO)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1327,44 +1327,44 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Jessica Cristina Macedo de Almeida</t>
+          <t>Jhully</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>+5531997424320</t>
+          <t>+5531991186576</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Rua Duque de Caxias 46 Casa A - portão de madeira, Betim</t>
+          <t>Rua Jonas Soares 235 Coopermapp, Contagem</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Aplique tic tac liso ou ondulado fibra Bio Orgânica Premium diversas cores*1</t>
+          <t>Kit 3/5/10 Calcinha Fio Dental Canelada Forro 100% Algodão Canelado Maju*1</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>39.53</t>
+          <t>0.53</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-06-08 12:21:48</t>
+          <t>2026-09-10 12:12:43</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6050226216656</t>
+          <t>3320030944939</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>(CTG LOC)BRUNO DINIZ SALES SILVA(NOVO)</t>
+          <t>(CTG LOC) ANDRESSA RAIANE MERCES(NOVO)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1374,44 +1374,44 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Adriana Rezende da Rocha</t>
+          <t>Raquel</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>+5531975448137</t>
+          <t>+5531991956627</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Av nossa senhora da paz Condomínio fazendinha são Miguel, São Joaquim de Bicas</t>
+          <t>Rua Gama 95 Bloco 28, apartamento 34, Contagem</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Vestido feminino*1</t>
+          <t>Saia Couro Fake Moda Verão*1</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>54.42</t>
+          <t>2.7</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-06-08 12:14:02</t>
+          <t>2026-09-10 12:12:38</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3320071483711</t>
+          <t>3320033940638</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>(CTG INT) Jessica Maiara da Silva</t>
+          <t>(CTG LOC) ANDRESSA RAIANE MERCES(NOVO)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1421,44 +1421,44 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>marcelacristinyro1</t>
+          <t>Lorena</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>+5531992651021</t>
+          <t>+5531999343903</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Rua Ronnie Peterson 447 condominio casa 6, Betim</t>
+          <t>Rua Doutor Olegário Ribeiro 43, Contagem</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Taba Squishy De Pintinho Fofo Brinquedo Alívio Estresse Apertar Bichinho Macio Brinquedo Antiestresse*1</t>
+          <t>Microfone de Lapela Sem Fio Profissional para Gravar Vídeo | Áudio Claro, Magnético e Bateria Duradoura vibration speaker*1</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.39</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-06-08 12:11:19</t>
+          <t>2026-09-10 12:11:57</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3320081477185</t>
+          <t>3320097947935</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Izabela Florencia(BIANCA MORAES)</t>
+          <t>(CTG LOC)Valdir Belmiro de Almeida</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1468,32 +1468,690 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Washington Santos</t>
+          <t>Maria Costa</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>+5531982455478</t>
+          <t>+5531998444566</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>rua Rio sacramento 790 casa, Contagem</t>
+          <t>Rua Geremias Alves 264 casa, Contagem</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Kit Masculino 6 Body Splash Famosos Nacionais e Arabes 60ml*1</t>
+          <t>Novo cinto feminino em formato de coração com corrente de diamantes 2024*1</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-06-08 12:11:06</t>
+          <t>2026-09-10 12:11:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>3320045943193</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>(CTG LOC) SAMUEL RONALD(NOVO)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Brunna lemes</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>+5531975223541</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Rua Rio Orenoco 276 Casa, Contagem</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Conjunto Mini Short saia e cropped casual Chic*1</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>57.9</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-09-10 12:11:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>3320012945611</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>(CTG LOC)TIAGO EUSTAQUIO S. CRUZ(NOVO)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>gabsf22x</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>+5531998190194</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Rua Durval de Souza Lima 129 apto 703, Contagem</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>SwanTears Máscara para Olhos (60 unidades) / Niacinamida, Cafeína, Peptídeos, Extratos Vegetais / Ilumina, reduz o inchaço, combate o envelhecimento e acalma a pele*1</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-09-10 12:11:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>3320002955587</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>(CTG LOC)CHRISTIAN WILLIAM J SILVA(NOVO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Izabelle Ferreira dos Santos Pinto</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>+5531989810892</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Rua Antônio Teixeira Ferraz 126 Casa, Contagem</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Conjunto Renda Conforto Abertura de Amarrar - Renda Delicada e Confortável com Amarração Ajustável para Melhor Encaixe e Elegância*1</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>11.91</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-09-10 12:10:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>3320053933656</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>(CTG LOC) ANDRESSA RAIANE MERCES(NOVO)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>cs</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>+5531973109403</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Avenida Coronel Benjamim Guimarães 1801 chamar por Tânia, Contagem</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Fone Bluetooth Sem Fio com Estojo | Conexão Rápida + Som Limpo*1</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>0.92</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-09-10 12:10:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>3320093934589</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>(CTG LOC) GABRIEL SABINO(SAULO SABINO)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Tiago</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>+5531991752021</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Rua São Geraldo 108 casa frente - telhado branco, Contagem</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>365 Hábitos Simples e Poderosos*1</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>16.56</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-09-10 12:09:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>3320059946036</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Janaina Santos (SAULO)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Luziane Karine</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>+5538998250799</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Rua Joaquim José 577 apt402 bl 01, Contagem</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Vestido Regata Feminina em linho com Forro zíper nas Costas Elegante com Fenda Lateral*1</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>17.97</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-09-10 12:09:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>3320080918758</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>(CTG LOC) Thiago antonio Alves</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Mariane</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>+5531996737158</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Rua José da Silva Couto 350, Contagem</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Mixer 600W Inox Elgin*1</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>107.99</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-09-10 09:41:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>6083026395231</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>(CTG LOC) Jessica Malta Ferrara(Thiago)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Leticia de Souza</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>+5531989556232</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Rua Padre Júlio Maria 60 Casa, Contagem</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>calças de tecido feminino*1</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>33.5</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:00:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>3320029930902</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>(CTG LOC) Luciene Maria Rodrigues</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Kennedy ferreira Rodrigues</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>+5531991292531</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Via de Acesso 675 mandar mensagem qnd chegar, Contagem</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Faixa Modeladora Feminina Alta Compressão Sinta Abdominal Plus Size Ajustável Confortável e Respirável Para Sair Treino Dia A Dia Moda Feminina*1</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>1.58</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-09-09 15:31:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>3320028915410</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>(LOC CTG) MARCIO MAGELA TEODORO (NOVO)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Júlia Silva</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>+5531973133805</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Rua Antônia Prates 144 casa, Contagem</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Kit Alongamento Gel + 100 Tips + Lixa + Mini Cabine De Unha + Pincel*1</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-09-09 15:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>3320061754627</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>(CTG INT) JOAQUIM CELESTINO(NOVO)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Valentina Silva Ottoni</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>+5531972165127</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Rua São João Evangelista s/n casa, Betim</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Estojo De Lápis De Grande Capacidade Camada Para Escolar*1</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>5.25</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-09-09 11:13:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>3320081909695</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>(CTG LOC) Talisson Fernando Ferreira(LK)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Deisiane Canuta</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>+5531975123399</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Rua Dezesseis 100 Casa, Contagem</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>12 Hastes Guarda Chuva Automático Sombrinha Grande Proteção Solar UV Reforçado Dobrável Envio Imediato colorido*1+12 Hastes Guarda Chuva Automático Sombrinha Grande Proteção Solar UV Reforçado Dobrável Envio Imediato colorido*1</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-09-09 11:12:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>3320027900301</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>(CTG LOC)CHRISTIAN WILLIAM J SILVA(NOVO</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Gilda Silva</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>+5531984274309</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Rua Vereador José Augusto Diniz 644 Casa, Bairro Santa Helena Contagem, Contagem</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Kit 5 Lâmpadas Super Bulbo Led 20w Branca Fria 6500k E27 Elgin*1</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>13.07</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-09-09 11:12:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>3320086869248</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>(CTG LOC) Eliomar Gomes Da Rocha</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Fake Delivery</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Viviane Carvalho De Souza</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>+5531994846549</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Rua Vista Alegre 126 Apt 401 bl06, Contagem</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Camisa Feminina Social Lisa Manga CURTA Botões Casual Elegante.*1</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>38.5</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:36:30</t>
         </is>
       </c>
     </row>

</xml_diff>